<commit_message>
Fix Union Boss Team 1 for max damage — no tanks
Union Boss is a damage race, not survival. Team 1 now matches
World Boss: Yord, Sera, Verna, Crystal, Monica (all back row).
Andrew/Dragonic reserved for PvP and UB Teams 2+.

Co-authored-by: Scurnow88 <Scurnow88@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/x-clash/X-CLASH-MASTER-RAW-DATA.xlsx
+++ b/x-clash/X-CLASH-MASTER-RAW-DATA.xlsx
@@ -428,7 +428,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Team 1 (Rally Leader)</t>
+          <t>Team 1 (Max Damage)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -496,22 +496,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Front</t>
+          <t>Back</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Andrew</t>
+          <t>Yord</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Tank</t>
+          <t>Buffer</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>~1.4M HP — absorbs boss hits for rally</t>
+          <t>Mandatory — team ATK/CRIT buff</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Team 1 (Rally Leader)</t>
+          <t>Team 1 (Max Damage)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Yord</t>
+          <t>Sera</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Mandatory team buffer</t>
+          <t>Forest faction + amplification</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Team 1 (Rally Leader)</t>
+          <t>Team 1 (Max Damage)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -585,17 +585,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sera</t>
+          <t>Verna</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Buffer</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Forest faction buff + heals</t>
+          <t>+17.45% monster DMG + boss debuff</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Team 1 (Rally Leader)</t>
+          <t>Team 1 (Max Damage)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -627,17 +627,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Verna</t>
+          <t>Crystal</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>Buffer/DPS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>+17.45% monster DMG (Astral Guardian)</t>
+          <t>Soul Protection buffs Monica + Verna</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Team 1 (Rally Leader)</t>
+          <t>Team 1 (Max Damage)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -669,17 +669,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Crystal</t>
+          <t>Monica</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Buffer/DPS</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Soul Protection buffs Forest back row</t>
+          <t>Forest crit DPS — no tanks (UB = max damage)</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Mandatory team buffer</t>
+          <t>Same lineup as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Forest faction + amplification</t>
+          <t>Same lineup as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Monster specialist — debuff + monster DMG amp</t>
+          <t>Same lineup as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Soul Protection buffs Monica + Verna</t>
+          <t>Same lineup as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Forest crit DPS — replaces Andrew (no tank on WB)</t>
+          <t>Same lineup as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="48" customWidth="1" min="17" max="17"/>
+    <col width="45" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1369,7 +1369,7 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>PvP front — reserve for UB/WB Team 2+</t>
+          <t>UB Team 2+ / PvP — tanks hurt boss damage</t>
         </is>
       </c>
     </row>
@@ -1421,11 +1421,7 @@
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
@@ -1440,7 +1436,7 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>UB Team 1 front only — not on WB (use Monica)</t>
+          <t>PvP front only — skip UB (damage mode)</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1507,7 @@
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PvP Human slot — WB alt if Monica locked elsewhere</t>
+          <t>UB Team 2+ / PvP Human DPS</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1634,11 @@
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>1</t>
@@ -1647,7 +1647,7 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>WB Team 1 DPS — replaces Andrew</t>
+          <t>UB + WB Team 1 DPS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise boss Team 1: drop Verna after user's WB results
User's Ancient Mammoth scores (1.1G–1.4G) used Yord + high-CP DPS,
not Verna. New Team 1: Yord, Sera, Monica, Crystal, Fenixia.
Verna benched on boss until CP/gear catches up; still PvP option.

Co-authored-by: Scurnow88 <Scurnow88@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/x-clash/X-CLASH-MASTER-RAW-DATA.xlsx
+++ b/x-clash/X-CLASH-MASTER-RAW-DATA.xlsx
@@ -428,7 +428,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Mandatory — team ATK/CRIT buff</t>
+          <t>Mandatory — in all your top WB scores (~1.1–1.4G)</t>
         </is>
       </c>
     </row>
@@ -548,12 +548,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Buffer</t>
+          <t>DPS/Buffer</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Forest faction + amplification</t>
+          <t>Highest CP — main damage + amplification</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Verna</t>
+          <t>Monica</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>+17.45% monster DMG + boss debuff</t>
+          <t>Forest crit burst — proven boss DPS</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Soul Protection buffs Monica + Verna</t>
+          <t>Soul Protection buffs Sera + Monica (Forest back row)</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Monica</t>
+          <t>Fenixia</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Forest crit DPS — no tanks (UB = max damage)</t>
+          <t>Human burst — 33/33/33; replaces Verna (underperformed)</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Same lineup as Union Boss Team 1</t>
+          <t>Same as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -758,12 +758,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Buffer</t>
+          <t>DPS/Buffer</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Same lineup as Union Boss Team 1</t>
+          <t>Same as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Verna</t>
+          <t>Monica</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Same lineup as Union Boss Team 1</t>
+          <t>Same as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Same lineup as Union Boss Team 1</t>
+          <t>Same as Union Boss Team 1</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Monica</t>
+          <t>Fenixia</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Same lineup as Union Boss Team 1</t>
+          <t>Same as Union Boss Team 1 — verified vs Verna on your account</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Forest — fine for PvP; benched on boss</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Human — swap Monica or Yord as needed</t>
+          <t>Human</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="45" customWidth="1" min="17" max="17"/>
+    <col width="48" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Core buffer — both boss modes</t>
+          <t>Team 1 core — highest CP damage carry</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>UB Team 2+ / PvP — tanks hurt boss damage</t>
+          <t>UB Team 2+ / PvP only</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PvP front only — skip UB (damage mode)</t>
+          <t>PvP front — skip boss teams</t>
         </is>
       </c>
     </row>
@@ -1492,8 +1492,16 @@
           <t>7</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>1</t>
@@ -1504,10 +1512,14 @@
           <t>S</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>UB Team 2+ / PvP Human DPS</t>
+          <t>Team 1 DPS — replaced Verna after WB testing</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1594,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Back-row Forest buff — both boss modes</t>
+          <t>Buffs Sera + Monica back row</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1669,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>UB + WB Team 1 DPS</t>
+          <t>Team 1 core DPS</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1744,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Mandatory buffer — both boss modes</t>
+          <t>Mandatory — in all top WB scores</t>
         </is>
       </c>
     </row>
@@ -1915,13 +1927,17 @@
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>4★ — not boss-ready</t>
+          <t>Ascend to 5★ — future boss DPS (see leaderboard meta)</t>
         </is>
       </c>
     </row>
@@ -2036,34 +2052,26 @@
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>SS+</t>
+          <t>D</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>SS+</t>
+          <t>F</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Boss specialist — both modes despite low CP</t>
+          <t>Benched boss — lowest CP; monster % kit needs heavy investment</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix boss Team 1: Kataras core from user's 1.4G WB run
Correct misidentification of lineup members and stale Aug stats.
Kataras was wrongly listed as low-skill tank; user confirmed best
WB score (1.4G rank 16) used Kataras. Team: Sera, Monica, Kataras,
Dragonic, Crystal (slots 1/4/5 need user confirm).

Co-authored-by: Scurnow88 <Scurnow88@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/x-clash/X-CLASH-MASTER-RAW-DATA.xlsx
+++ b/x-clash/X-CLASH-MASTER-RAW-DATA.xlsx
@@ -501,17 +501,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Yord</t>
+          <t>Sera</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Buffer</t>
+          <t>DPS/Buffer</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Mandatory — in all your top WB scores (~1.1–1.4G)</t>
+          <t>Forest DPS — slot 1 in your 1.4G WB run (rank 16)</t>
         </is>
       </c>
     </row>
@@ -543,17 +543,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sera</t>
+          <t>Monica</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>DPS/Buffer</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Highest CP — main damage + amplification</t>
+          <t>Forest DPS — slot 2 in 1.4G run</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Monica</t>
+          <t>Kataras</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Forest crit burst — proven boss DPS</t>
+          <t>Your highest WB score (1.4G) — core pick; NOT Yord</t>
         </is>
       </c>
     </row>
@@ -622,22 +622,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Back</t>
+          <t>Front</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Crystal</t>
+          <t>Dragonic</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Buffer/DPS</t>
+          <t>Tank/DPS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Soul Protection buffs Sera + Monica (Forest back row)</t>
+          <t>Demon front — in 1.4G run; your data beats no-tank theory</t>
         </is>
       </c>
     </row>
@@ -669,17 +669,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Fenixia</t>
+          <t>Crystal</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>Buffer/DPS</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Human burst — 33/33/33; replaces Verna (underperformed)</t>
+          <t>Mage/support slot in 1.4G run — Forest back-row buff</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team 1 (Verified Best)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -711,17 +711,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Yord</t>
+          <t>Sera</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Buffer</t>
+          <t>DPS/Buffer</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Same as Union Boss Team 1</t>
+          <t>1.4G Ancient Mammoth — CP 18.6M team</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team 1 (Verified Best)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -753,17 +753,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sera</t>
+          <t>Monica</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>DPS/Buffer</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Same as Union Boss Team 1</t>
+          <t>1.4G run rank 16</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team 1 (Verified Best)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Monica</t>
+          <t>Kataras</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Same as Union Boss Team 1</t>
+          <t>User confirmed — best WB performer</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team 1 (Verified Best)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -832,22 +832,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Back</t>
+          <t>Front</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Crystal</t>
+          <t>Dragonic</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Buffer/DPS</t>
+          <t>Tank/DPS</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Same as Union Boss Team 1</t>
+          <t>1.4G run — demon/tank slot</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team 1 (Verified Best)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -879,17 +879,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Fenixia</t>
+          <t>Crystal</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>Buffer/DPS</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Same as Union Boss Team 1 — verified vs Verna on your account</t>
+          <t>1.4G run — confirm in-game if different</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Forest — fine for PvP; benched on boss</t>
+          <t>Forest — PvP only</t>
         </is>
       </c>
     </row>
@@ -1118,8 +1118,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Team 1 core — highest CP damage carry</t>
+          <t>WB 1.4G run slot 1 — Aug stats; likely higher now (Lv150)</t>
         </is>
       </c>
     </row>
@@ -1354,8 +1354,16 @@
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>1</t>
@@ -1366,10 +1374,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>UB Team 2+ / PvP only</t>
+          <t>WB 1.4G run front — demon slot; Aug stats stale</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1448,7 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PvP front — skip boss teams</t>
+          <t>PvP front only</t>
         </is>
       </c>
     </row>
@@ -1492,21 +1504,9 @@
           <t>7</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
           <t>S</t>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Team 1 DPS — replaced Verna after WB testing</t>
+          <t>Strong DPS but not in your 1.4G best run</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Buffs Sera + Monica back row</t>
+          <t>WB 1.4G run slot 5 — confirm in-game</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Team 1 core DPS</t>
+          <t>WB 1.4G run slot 2</t>
         </is>
       </c>
     </row>
@@ -1721,16 +1721,8 @@
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
@@ -1739,12 +1731,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Mandatory — in all top WB scores</t>
+          <t>Not in 1.4G best run — optional buffer not core for you</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1799,7 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Reserve — low skills</t>
+          <t>Reserve</t>
         </is>
       </c>
     </row>
@@ -1819,17 +1811,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>The Guardian</t>
+          <t>Demon Masked Asura</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nightfall</t>
+          <t>God/Nightfall</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tank</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1859,18 +1851,30 @@
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+          <t>SS+</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SS+</t>
+        </is>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Reserve — low skills</t>
+          <t>BEST WB score 1.4G — was mislabeled tank; Aug skill lv stale (now Lv150)</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1941,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Ascend to 5★ — future boss DPS (see leaderboard meta)</t>
+          <t>May be slot 1 in 1.4G run — confirm vs Sera</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2004,7 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>3★ — not boss-ready</t>
+          <t>May be slot 4 demon — confirm vs Dragonic</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2065,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -2071,7 +2075,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Benched boss — lowest CP; monster % kit needs heavy investment</t>
+          <t>Benched boss — user verified poor WB damage</t>
         </is>
       </c>
     </row>
@@ -2770,12 +2774,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>PvP</t>
+          <t>PvP / World Boss</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -2790,12 +2794,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Belial / Mirana</t>
+          <t>Belial / Mirana / Monica</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Verify faction in-game</t>
+          <t>Verify faction in-game; user WB 1.4G with Kataras</t>
         </is>
       </c>
     </row>

</xml_diff>